<commit_message>
2026, 2027 images added, some locations images added
</commit_message>
<xml_diff>
--- a/data/Locations.xlsx
+++ b/data/Locations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\landscapingUOB-api\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E5B1A2E-5A24-401C-A2D6-EA83994DD2ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A98D4AEE-B9BD-48DF-9BC7-7CE0E90A0793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="162">
   <si>
     <t>Location type</t>
   </si>
@@ -182,9 +182,6 @@
     <t>Deanship of Admission &amp; Registration</t>
   </si>
   <si>
-    <t>https://i.postimg.cc/MT3Ywv7H/S37-1.jpg</t>
-  </si>
-  <si>
     <t>S38</t>
   </si>
   <si>
@@ -368,9 +365,6 @@
     <t>Mosque</t>
   </si>
   <si>
-    <t>https://i.postimg.cc/G2PN8NJ4/Buildings-image.png</t>
-  </si>
-  <si>
     <t>Infrastructure</t>
   </si>
   <si>
@@ -380,9 +374,6 @@
     <t>Boundary Wall</t>
   </si>
   <si>
-    <t>https://i.postimg.cc/bwr6y42y/Boundary-wall.jpg</t>
-  </si>
-  <si>
     <t>Facilities</t>
   </si>
   <si>
@@ -462,6 +453,75 @@
   </si>
   <si>
     <t>https://i.postimg.cc/PJXwkWyR/In_front_of_S45_7.jpg</t>
+  </si>
+  <si>
+    <t>Image 4</t>
+  </si>
+  <si>
+    <t>Image 5</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/L6603kBS/S17-4.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/wTTbQ5c3/S17-3.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/vHHSt7LT/S17-2.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/YqqyzNfH/S17-area3.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/DzVk693V/DSC-0114.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/FH3Yqd05/S1A-4.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/RFQ8bRZQ/S1B-2.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/cH4j23t0/S2-Surroundings-4.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/TwYSFb5G/S2-Surroundings-2.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/V6sVVmqm/infrastructure.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/4xgyHSvr/S6.png</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/wBVctNSJ/S22-6.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/Jh1YdRm7/S37-6.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/25z9XCmk/S37.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/nL0RyNcb/S37-1.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/ZKWWpNyg/S38-3.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/9FDDZ9qn/S38-6-(1).jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/59hX50q1/S39-5.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/v8J47BLy/S39-7.jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/xjwXGCy2/S39-5-(1).jpg</t>
+  </si>
+  <si>
+    <t>https://i.postimg.cc/wxC15vc6/S39-3.jpg</t>
   </si>
 </sst>
 </file>
@@ -854,7 +914,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.90625" customWidth="1"/>
@@ -862,17 +922,19 @@
     <col min="3" max="3" width="53.36328125" customWidth="1"/>
     <col min="4" max="4" width="46.453125" style="4" customWidth="1"/>
     <col min="5" max="5" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="44.36328125" customWidth="1"/>
-    <col min="7" max="7" width="45.1796875" customWidth="1"/>
-    <col min="8" max="8" width="46" customWidth="1"/>
+    <col min="6" max="6" width="41.90625" customWidth="1"/>
+    <col min="7" max="7" width="44.81640625" customWidth="1"/>
+    <col min="8" max="8" width="46.1796875" customWidth="1"/>
+    <col min="9" max="9" width="38.36328125" customWidth="1"/>
+    <col min="10" max="10" width="38.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -881,19 +943,25 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -909,8 +977,23 @@
       <c r="E2">
         <v>699</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F2" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="H2" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="I2" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="J2" s="13" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -926,8 +1009,14 @@
       <c r="E3">
         <v>600</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F3" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="13" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -943,8 +1032,14 @@
       <c r="E4">
         <v>350</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F4" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -960,8 +1055,14 @@
       <c r="E5">
         <v>186</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F5" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -977,8 +1078,17 @@
       <c r="E6">
         <v>77</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -994,8 +1104,11 @@
       <c r="E7">
         <v>330</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F7" s="13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1011,8 +1124,11 @@
       <c r="E8">
         <v>280</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F8" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -1028,8 +1144,11 @@
       <c r="E9">
         <v>270</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F9" s="13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -1045,8 +1164,11 @@
       <c r="E10">
         <v>120</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F10" s="13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -1062,8 +1184,14 @@
       <c r="E11">
         <v>440</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F11" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>3</v>
       </c>
@@ -1079,8 +1207,11 @@
       <c r="E12">
         <v>105</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F12" s="13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>3</v>
       </c>
@@ -1096,8 +1227,11 @@
       <c r="E13">
         <v>1050</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F13" s="13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>3</v>
       </c>
@@ -1113,8 +1247,11 @@
       <c r="E14">
         <v>80</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F14" s="13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>3</v>
       </c>
@@ -1130,8 +1267,11 @@
       <c r="E15">
         <v>145</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F15" s="13" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>3</v>
       </c>
@@ -1142,285 +1282,318 @@
         <v>47</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>48</v>
+        <v>153</v>
       </c>
       <c r="E16">
         <v>1350</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F16" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="H16" s="13" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>3</v>
       </c>
       <c r="B17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" t="s">
         <v>49</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>51</v>
       </c>
       <c r="E17">
         <v>175</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F17" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="H17" s="13" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>3</v>
       </c>
       <c r="B18" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" t="s">
         <v>52</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>54</v>
       </c>
       <c r="E18">
         <v>1000</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="F18" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="G18" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="J18" s="13" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
         <v>3</v>
       </c>
       <c r="B19" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="8" t="s">
         <v>56</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>57</v>
       </c>
       <c r="E19" s="7">
         <v>1000</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>3</v>
       </c>
       <c r="B20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" t="s">
         <v>58</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>60</v>
       </c>
       <c r="E20">
         <v>350</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>3</v>
       </c>
       <c r="B21" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" t="s">
         <v>61</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>63</v>
       </c>
       <c r="E21">
         <v>464</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>3</v>
       </c>
       <c r="B22" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" t="s">
         <v>64</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>66</v>
       </c>
       <c r="E22">
         <v>310</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>3</v>
       </c>
       <c r="B23" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" t="s">
         <v>67</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>69</v>
       </c>
       <c r="E23">
         <v>195</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>3</v>
       </c>
       <c r="B24" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" t="s">
         <v>70</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" s="5" t="s">
         <v>71</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>72</v>
       </c>
       <c r="E24">
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>3</v>
       </c>
       <c r="B25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" t="s">
         <v>73</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>75</v>
       </c>
       <c r="E25">
         <v>180</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>3</v>
       </c>
       <c r="B26" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" t="s">
         <v>76</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>78</v>
       </c>
       <c r="E26">
         <v>90</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H26" s="13" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>3</v>
       </c>
       <c r="B27" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" t="s">
         <v>79</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" s="5" t="s">
         <v>80</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>81</v>
       </c>
       <c r="E27">
         <v>150</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="7" t="s">
         <v>3</v>
       </c>
       <c r="B28" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="D28" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="D28" s="8" t="s">
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>3</v>
-      </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>85</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" s="5" t="s">
         <v>86</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>87</v>
       </c>
       <c r="E29">
         <v>399</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>3</v>
       </c>
       <c r="B30" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" t="s">
         <v>88</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" s="5" t="s">
         <v>89</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>90</v>
       </c>
       <c r="E30">
         <v>163</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>3</v>
       </c>
       <c r="B31" t="s">
+        <v>90</v>
+      </c>
+      <c r="C31" t="s">
         <v>91</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>93</v>
       </c>
       <c r="E31">
         <v>194</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>3</v>
       </c>
       <c r="B32" t="s">
+        <v>93</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="D32" s="5" t="s">
         <v>95</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>96</v>
       </c>
       <c r="E32">
         <v>373</v>
@@ -1431,13 +1604,13 @@
         <v>3</v>
       </c>
       <c r="B33" t="s">
+        <v>96</v>
+      </c>
+      <c r="C33" t="s">
+        <v>88</v>
+      </c>
+      <c r="D33" s="5" t="s">
         <v>97</v>
-      </c>
-      <c r="C33" t="s">
-        <v>89</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="E33">
         <v>161</v>
@@ -1448,13 +1621,13 @@
         <v>3</v>
       </c>
       <c r="B34" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C34" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="D34" s="8" t="s">
         <v>100</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>101</v>
       </c>
       <c r="E34" s="7">
         <v>600</v>
@@ -1465,13 +1638,13 @@
         <v>3</v>
       </c>
       <c r="B35" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="D35" s="8" t="s">
         <v>103</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>104</v>
       </c>
       <c r="E35" s="7">
         <v>205</v>
@@ -1482,13 +1655,13 @@
         <v>3</v>
       </c>
       <c r="B36" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="D36" s="8" t="s">
         <v>106</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>107</v>
       </c>
       <c r="E36" s="7">
         <v>205</v>
@@ -1499,13 +1672,13 @@
         <v>3</v>
       </c>
       <c r="B37" t="s">
+        <v>107</v>
+      </c>
+      <c r="C37" t="s">
         <v>108</v>
       </c>
-      <c r="C37" t="s">
-        <v>109</v>
-      </c>
       <c r="D37" s="5" t="s">
-        <v>110</v>
+        <v>151</v>
       </c>
       <c r="E37">
         <v>350</v>
@@ -1513,16 +1686,16 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C38" t="s">
         <v>111</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="C38" t="s">
-        <v>113</v>
-      </c>
       <c r="D38" s="5" t="s">
-        <v>114</v>
+        <v>150</v>
       </c>
       <c r="E38">
         <v>142</v>
@@ -1530,13 +1703,13 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B39" t="s">
         <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D39" s="9"/>
       <c r="E39">
@@ -1545,16 +1718,16 @@
     </row>
     <row r="40" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B40" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D40" s="8" t="s">
         <v>115</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>118</v>
       </c>
       <c r="E40" s="7">
         <v>600</v>
@@ -1562,16 +1735,16 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
+        <v>116</v>
+      </c>
+      <c r="B41" t="s">
+        <v>117</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D41" s="5" t="s">
         <v>119</v>
-      </c>
-      <c r="B41" t="s">
-        <v>120</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>122</v>
       </c>
       <c r="E41">
         <v>5300</v>
@@ -1579,16 +1752,16 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B42" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C42" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E42">
         <v>16500</v>
@@ -1596,16 +1769,16 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B43" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C43" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E43">
         <v>16500</v>
@@ -1613,7 +1786,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B44" t="s">
         <v>25</v>
@@ -1630,16 +1803,16 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B45" t="s">
+        <v>51</v>
+      </c>
+      <c r="C45" t="s">
         <v>52</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" s="5" t="s">
         <v>53</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>54</v>
       </c>
       <c r="E45">
         <v>400</v>
@@ -1647,16 +1820,16 @@
     </row>
     <row r="46" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="7" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B46" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C46" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C46" s="7" t="s">
+      <c r="D46" s="8" t="s">
         <v>56</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>57</v>
       </c>
       <c r="E46" s="7">
         <v>400</v>
@@ -1664,16 +1837,16 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B47" t="s">
+        <v>60</v>
+      </c>
+      <c r="C47" t="s">
         <v>61</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>63</v>
       </c>
       <c r="E47">
         <v>704</v>
@@ -1681,16 +1854,16 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B48" t="s">
+        <v>63</v>
+      </c>
+      <c r="C48" t="s">
         <v>64</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>66</v>
       </c>
       <c r="E48">
         <v>602</v>
@@ -1698,16 +1871,16 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C49" t="s">
         <v>82</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>84</v>
       </c>
       <c r="E49">
         <v>128</v>
@@ -1715,16 +1888,16 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B50" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C50" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E50">
         <v>825</v>
@@ -1738,7 +1911,7 @@
         <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D51" s="10"/>
       <c r="E51">
@@ -1747,11 +1920,11 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B52" s="11"/>
       <c r="C52" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D52" s="10"/>
       <c r="E52">
@@ -1771,56 +1944,90 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="D5" r:id="rId1" xr:uid="{80EE9128-EF22-45E1-A050-B4A922D7A5A4}"/>
-    <hyperlink ref="D25" r:id="rId2" xr:uid="{CA6F2ACE-9B39-4D45-9C20-19A5DB6D12CA}"/>
-    <hyperlink ref="D15" r:id="rId3" xr:uid="{892A1EEC-B028-4BF1-ADCD-AF96A0988B50}"/>
-    <hyperlink ref="D10" r:id="rId4" xr:uid="{F1426B06-7CBB-4D59-AE83-B095FA6474E2}"/>
-    <hyperlink ref="D8" r:id="rId5" xr:uid="{592D78FC-336C-471A-91BD-1562E94DA284}"/>
-    <hyperlink ref="D9" r:id="rId6" xr:uid="{A2D386D9-0502-4921-BB61-A819FF837370}"/>
-    <hyperlink ref="D19" r:id="rId7" xr:uid="{7BE3DA68-E823-4B16-885B-945823145A4E}"/>
-    <hyperlink ref="D13" r:id="rId8" xr:uid="{5A89EF2A-F868-480F-9E72-4F25C74088A4}"/>
-    <hyperlink ref="D31" r:id="rId9" xr:uid="{99947C2E-DEFB-4F3D-B10B-4C51E1A36A2A}"/>
-    <hyperlink ref="D33" r:id="rId10" xr:uid="{8D11C5C3-9012-49EE-A7E5-072DFCD7E4CB}"/>
-    <hyperlink ref="D2" r:id="rId11" xr:uid="{6CF4DEC1-CD4E-4844-A06E-A3B5553E4A0A}"/>
-    <hyperlink ref="D3" r:id="rId12" xr:uid="{9E806015-46CC-43F4-B15B-0F80E18DD0D3}"/>
-    <hyperlink ref="D4" r:id="rId13" xr:uid="{0BE1B822-D34C-40EF-8B0F-F98C95A68F23}"/>
-    <hyperlink ref="D11" r:id="rId14" xr:uid="{BD02D7C7-CF92-4415-BD68-A5E1CD860AB5}"/>
-    <hyperlink ref="D16" r:id="rId15" xr:uid="{B21EE433-AA31-44F8-A2B5-B896D27134D4}"/>
-    <hyperlink ref="D14" r:id="rId16" xr:uid="{E2D6E56A-BEDF-4371-A57A-AE46E0B0D271}"/>
-    <hyperlink ref="D17" r:id="rId17" xr:uid="{6EEDF604-934E-4BBF-844F-1CBB5949AF7F}"/>
-    <hyperlink ref="D18" r:id="rId18" xr:uid="{2D6E9249-18AB-4397-B0F5-437EFBC6F332}"/>
-    <hyperlink ref="D36" r:id="rId19" xr:uid="{E63D41F9-5B08-43E0-8053-0724E6D37B6B}"/>
-    <hyperlink ref="D21" r:id="rId20" xr:uid="{5BA1C18C-D565-4734-9906-9C0A7DC7BFEA}"/>
-    <hyperlink ref="D27" r:id="rId21" xr:uid="{40D3F8D6-8B9A-4507-8102-4BFB0D9B2580}"/>
-    <hyperlink ref="D26" r:id="rId22" xr:uid="{EFEDD41E-1E02-461C-9393-AD2ACCBC2A60}"/>
-    <hyperlink ref="D32" r:id="rId23" xr:uid="{0BEBBA09-865C-426C-A4B4-4F2481A2A4E8}"/>
-    <hyperlink ref="D12" r:id="rId24" xr:uid="{9B82FEF9-0E16-4B92-A3E1-1FC2CB2AF171}"/>
-    <hyperlink ref="D7" r:id="rId25" xr:uid="{2ED0409A-8763-4061-A855-6C9AC6A9D6BD}"/>
-    <hyperlink ref="D28" r:id="rId26" xr:uid="{A6B3F117-56EC-4411-89C5-2B81B32C6D2F}"/>
-    <hyperlink ref="D29" r:id="rId27" xr:uid="{45AB639A-6A68-47E6-820F-5AE96EF37CCE}"/>
-    <hyperlink ref="D30" r:id="rId28" xr:uid="{7CB307A7-AD29-447B-B87B-FDF01946BA4A}"/>
-    <hyperlink ref="D24" r:id="rId29" xr:uid="{D83D9F73-94C9-4362-9F33-9764794F83C7}"/>
-    <hyperlink ref="D23" r:id="rId30" xr:uid="{13D49606-5D63-4601-9617-2606341647E2}"/>
-    <hyperlink ref="D34" r:id="rId31" xr:uid="{E93DF50E-6385-47B4-B2C7-B9246E51EFC3}"/>
-    <hyperlink ref="D40" r:id="rId32" xr:uid="{887D03B3-F5B5-4EC3-B378-CFF1ACACC697}"/>
-    <hyperlink ref="D41" r:id="rId33" xr:uid="{25328B39-D4E0-444C-9000-8F992DB7BA09}"/>
-    <hyperlink ref="D20" r:id="rId34" xr:uid="{80ECF8CD-7A79-402A-B5EC-F9BA63C3B50A}"/>
-    <hyperlink ref="D43" r:id="rId35" xr:uid="{6B7E0906-BF85-4BF1-A5E5-9F4F8AB12E12}"/>
-    <hyperlink ref="D42" r:id="rId36" xr:uid="{A757999D-BA12-4BC4-B318-11BE5E932894}"/>
-    <hyperlink ref="D38" r:id="rId37" xr:uid="{6AF44C4C-D5AE-4BD7-8C44-C3D0460467C0}"/>
-    <hyperlink ref="D35" r:id="rId38" xr:uid="{368C86F0-6C72-4FCF-9F6B-86FBA36B83AF}"/>
-    <hyperlink ref="D6" r:id="rId39" xr:uid="{705A06BF-AD9E-4AEF-8BEC-6580A15197D6}"/>
-    <hyperlink ref="D37" r:id="rId40" xr:uid="{6683E2F8-FB9A-4014-9996-7FEAAC683B93}"/>
-    <hyperlink ref="D44" r:id="rId41" xr:uid="{F581F61C-236D-49A3-AE06-C2A7FF968C89}"/>
-    <hyperlink ref="D45" r:id="rId42" xr:uid="{BB91F514-736D-4FC9-A32E-788A20E577B9}"/>
-    <hyperlink ref="D46" r:id="rId43" xr:uid="{7EBDAD46-1A5B-4B2C-AF3D-61F18C3E275F}"/>
-    <hyperlink ref="D47" r:id="rId44" xr:uid="{A36D56AA-7C90-4154-A870-DA9409189D1F}"/>
-    <hyperlink ref="D22" r:id="rId45" xr:uid="{6E85802D-CC4C-4BD4-83ED-55100DE115BA}"/>
-    <hyperlink ref="D48" r:id="rId46" xr:uid="{00DDF648-5623-4E1D-8FC4-42D38FAEE4CA}"/>
-    <hyperlink ref="D49" r:id="rId47" xr:uid="{77EAAAD6-086C-4DCF-9B24-E59430A2E2FB}"/>
-    <hyperlink ref="D50" r:id="rId48" xr:uid="{CE8A3876-BF7A-4C23-95FB-161481F8F980}"/>
-    <hyperlink ref="F26" r:id="rId49" xr:uid="{E4CD215B-218A-44EC-9945-5F6AD197B3B2}"/>
-    <hyperlink ref="G26" r:id="rId50" xr:uid="{522CE0D5-7681-455E-9A32-6774CD570260}"/>
-    <hyperlink ref="H26" r:id="rId51" xr:uid="{A440C7F8-BC12-4ED8-80D1-5687F587FDDF}"/>
+    <hyperlink ref="D15" r:id="rId2" xr:uid="{892A1EEC-B028-4BF1-ADCD-AF96A0988B50}"/>
+    <hyperlink ref="D10" r:id="rId3" xr:uid="{F1426B06-7CBB-4D59-AE83-B095FA6474E2}"/>
+    <hyperlink ref="D8" r:id="rId4" xr:uid="{592D78FC-336C-471A-91BD-1562E94DA284}"/>
+    <hyperlink ref="D9" r:id="rId5" xr:uid="{A2D386D9-0502-4921-BB61-A819FF837370}"/>
+    <hyperlink ref="D13" r:id="rId6" xr:uid="{5A89EF2A-F868-480F-9E72-4F25C74088A4}"/>
+    <hyperlink ref="D2" r:id="rId7" xr:uid="{6CF4DEC1-CD4E-4844-A06E-A3B5553E4A0A}"/>
+    <hyperlink ref="D3" r:id="rId8" xr:uid="{9E806015-46CC-43F4-B15B-0F80E18DD0D3}"/>
+    <hyperlink ref="D4" r:id="rId9" xr:uid="{0BE1B822-D34C-40EF-8B0F-F98C95A68F23}"/>
+    <hyperlink ref="D11" r:id="rId10" xr:uid="{BD02D7C7-CF92-4415-BD68-A5E1CD860AB5}"/>
+    <hyperlink ref="D14" r:id="rId11" xr:uid="{E2D6E56A-BEDF-4371-A57A-AE46E0B0D271}"/>
+    <hyperlink ref="D12" r:id="rId12" xr:uid="{9B82FEF9-0E16-4B92-A3E1-1FC2CB2AF171}"/>
+    <hyperlink ref="D7" r:id="rId13" xr:uid="{2ED0409A-8763-4061-A855-6C9AC6A9D6BD}"/>
+    <hyperlink ref="D40" r:id="rId14" xr:uid="{887D03B3-F5B5-4EC3-B378-CFF1ACACC697}"/>
+    <hyperlink ref="D41" r:id="rId15" xr:uid="{25328B39-D4E0-444C-9000-8F992DB7BA09}"/>
+    <hyperlink ref="D43" r:id="rId16" xr:uid="{6B7E0906-BF85-4BF1-A5E5-9F4F8AB12E12}"/>
+    <hyperlink ref="D42" r:id="rId17" xr:uid="{A757999D-BA12-4BC4-B318-11BE5E932894}"/>
+    <hyperlink ref="D6" r:id="rId18" xr:uid="{705A06BF-AD9E-4AEF-8BEC-6580A15197D6}"/>
+    <hyperlink ref="D44" r:id="rId19" xr:uid="{F581F61C-236D-49A3-AE06-C2A7FF968C89}"/>
+    <hyperlink ref="D45" r:id="rId20" xr:uid="{BB91F514-736D-4FC9-A32E-788A20E577B9}"/>
+    <hyperlink ref="D46" r:id="rId21" xr:uid="{7EBDAD46-1A5B-4B2C-AF3D-61F18C3E275F}"/>
+    <hyperlink ref="D47" r:id="rId22" xr:uid="{A36D56AA-7C90-4154-A870-DA9409189D1F}"/>
+    <hyperlink ref="D48" r:id="rId23" xr:uid="{00DDF648-5623-4E1D-8FC4-42D38FAEE4CA}"/>
+    <hyperlink ref="D49" r:id="rId24" xr:uid="{77EAAAD6-086C-4DCF-9B24-E59430A2E2FB}"/>
+    <hyperlink ref="D50" r:id="rId25" xr:uid="{CE8A3876-BF7A-4C23-95FB-161481F8F980}"/>
+    <hyperlink ref="F26" r:id="rId26" xr:uid="{E4CD215B-218A-44EC-9945-5F6AD197B3B2}"/>
+    <hyperlink ref="G26" r:id="rId27" xr:uid="{522CE0D5-7681-455E-9A32-6774CD570260}"/>
+    <hyperlink ref="H26" r:id="rId28" xr:uid="{A440C7F8-BC12-4ED8-80D1-5687F587FDDF}"/>
+    <hyperlink ref="G2" r:id="rId29" xr:uid="{E92EE150-871A-439E-974B-FA2049C8CA38}"/>
+    <hyperlink ref="H2" r:id="rId30" xr:uid="{03D46786-9004-478B-A395-4AA7EF082A56}"/>
+    <hyperlink ref="I2" r:id="rId31" xr:uid="{57A7AAAC-E898-44F4-A3B0-AF97E1EBFE69}"/>
+    <hyperlink ref="J2" r:id="rId32" xr:uid="{ACBBE8A2-CC26-4054-A6DA-6E5C07960AD1}"/>
+    <hyperlink ref="F3" r:id="rId33" xr:uid="{29114336-215A-43FA-8297-CDDD761C1501}"/>
+    <hyperlink ref="G3" r:id="rId34" xr:uid="{0AE835A0-8DDB-4A91-8176-2AFF9C2AEA07}"/>
+    <hyperlink ref="F4" r:id="rId35" xr:uid="{9F1D3B58-9986-4688-ABF5-8FF2375FBF82}"/>
+    <hyperlink ref="G4" r:id="rId36" xr:uid="{6CB43155-6638-4798-B491-DB6FA525EB50}"/>
+    <hyperlink ref="F5" r:id="rId37" xr:uid="{7DCFF457-0664-4586-B064-437E516400A0}"/>
+    <hyperlink ref="G5" r:id="rId38" xr:uid="{343CFCD0-DE46-476D-8E81-253A8E3B316C}"/>
+    <hyperlink ref="F6" r:id="rId39" xr:uid="{3EC21E9D-842C-4CB8-B811-D23F2C778BF7}"/>
+    <hyperlink ref="G6" r:id="rId40" xr:uid="{33FCB128-9197-43CE-8CB7-FE8F3059BE4F}"/>
+    <hyperlink ref="H6" r:id="rId41" xr:uid="{1F8966A1-2290-4CEF-BB02-FC990CD8D791}"/>
+    <hyperlink ref="F7" r:id="rId42" xr:uid="{423CFF82-45DF-4D68-BB50-979F20779C0F}"/>
+    <hyperlink ref="F8" r:id="rId43" xr:uid="{E5CBA92A-AB4F-478A-9CFE-9419577F0ED5}"/>
+    <hyperlink ref="F10" r:id="rId44" xr:uid="{EB116F53-35BE-4168-A3B3-A6B7F3013480}"/>
+    <hyperlink ref="F9" r:id="rId45" xr:uid="{AAFC07D3-B9CC-483D-8F88-4D08FD7ED6B1}"/>
+    <hyperlink ref="F11" r:id="rId46" xr:uid="{E9FA1CD4-77B0-4337-B7D9-41FF5FAF8D5C}"/>
+    <hyperlink ref="G11" r:id="rId47" xr:uid="{44406BDF-4864-4DEE-8D3F-960771AC5EEA}"/>
+    <hyperlink ref="F12" r:id="rId48" xr:uid="{A2470070-51EF-4670-833B-8D482C601671}"/>
+    <hyperlink ref="F13" r:id="rId49" xr:uid="{4D4972B4-0A24-4319-992B-3F7B5C4CCDCE}"/>
+    <hyperlink ref="F14" r:id="rId50" xr:uid="{AE1ACB1F-F85D-4CF3-AC72-FD2F25C8E4B2}"/>
+    <hyperlink ref="D22" r:id="rId51" xr:uid="{6E85802D-CC4C-4BD4-83ED-55100DE115BA}"/>
+    <hyperlink ref="D37" r:id="rId52" xr:uid="{6683E2F8-FB9A-4014-9996-7FEAAC683B93}"/>
+    <hyperlink ref="D35" r:id="rId53" xr:uid="{368C86F0-6C72-4FCF-9F6B-86FBA36B83AF}"/>
+    <hyperlink ref="D38" r:id="rId54" xr:uid="{6AF44C4C-D5AE-4BD7-8C44-C3D0460467C0}"/>
+    <hyperlink ref="D20" r:id="rId55" xr:uid="{80ECF8CD-7A79-402A-B5EC-F9BA63C3B50A}"/>
+    <hyperlink ref="D34" r:id="rId56" xr:uid="{E93DF50E-6385-47B4-B2C7-B9246E51EFC3}"/>
+    <hyperlink ref="D23" r:id="rId57" xr:uid="{13D49606-5D63-4601-9617-2606341647E2}"/>
+    <hyperlink ref="D24" r:id="rId58" xr:uid="{D83D9F73-94C9-4362-9F33-9764794F83C7}"/>
+    <hyperlink ref="D30" r:id="rId59" xr:uid="{7CB307A7-AD29-447B-B87B-FDF01946BA4A}"/>
+    <hyperlink ref="D29" r:id="rId60" xr:uid="{45AB639A-6A68-47E6-820F-5AE96EF37CCE}"/>
+    <hyperlink ref="D28" r:id="rId61" xr:uid="{A6B3F117-56EC-4411-89C5-2B81B32C6D2F}"/>
+    <hyperlink ref="D32" r:id="rId62" xr:uid="{0BEBBA09-865C-426C-A4B4-4F2481A2A4E8}"/>
+    <hyperlink ref="D26" r:id="rId63" xr:uid="{EFEDD41E-1E02-461C-9393-AD2ACCBC2A60}"/>
+    <hyperlink ref="D27" r:id="rId64" xr:uid="{40D3F8D6-8B9A-4507-8102-4BFB0D9B2580}"/>
+    <hyperlink ref="D21" r:id="rId65" xr:uid="{5BA1C18C-D565-4734-9906-9C0A7DC7BFEA}"/>
+    <hyperlink ref="D36" r:id="rId66" xr:uid="{E63D41F9-5B08-43E0-8053-0724E6D37B6B}"/>
+    <hyperlink ref="D18" r:id="rId67" xr:uid="{2D6E9249-18AB-4397-B0F5-437EFBC6F332}"/>
+    <hyperlink ref="D17" r:id="rId68" xr:uid="{6EEDF604-934E-4BBF-844F-1CBB5949AF7F}"/>
+    <hyperlink ref="D16" r:id="rId69" xr:uid="{B21EE433-AA31-44F8-A2B5-B896D27134D4}"/>
+    <hyperlink ref="D33" r:id="rId70" xr:uid="{8D11C5C3-9012-49EE-A7E5-072DFCD7E4CB}"/>
+    <hyperlink ref="D31" r:id="rId71" xr:uid="{99947C2E-DEFB-4F3D-B10B-4C51E1A36A2A}"/>
+    <hyperlink ref="D19" r:id="rId72" xr:uid="{7BE3DA68-E823-4B16-885B-945823145A4E}"/>
+    <hyperlink ref="D25" r:id="rId73" xr:uid="{CA6F2ACE-9B39-4D45-9C20-19A5DB6D12CA}"/>
+    <hyperlink ref="F15" r:id="rId74" xr:uid="{C35D8A0A-F10A-40F3-A7C3-C5AA6BBB28B5}"/>
+    <hyperlink ref="F16" r:id="rId75" xr:uid="{AEA8472C-440C-4C92-8A77-FEF9C839BF0D}"/>
+    <hyperlink ref="G16" r:id="rId76" xr:uid="{D288EC2B-5C10-4124-87EF-58A40C745452}"/>
+    <hyperlink ref="H16" r:id="rId77" xr:uid="{AB6F38F4-9CD4-49B8-9315-6A116F3871B3}"/>
+    <hyperlink ref="G17" r:id="rId78" xr:uid="{A5B70704-22DA-478D-9DD9-DCC7AA836C2E}"/>
+    <hyperlink ref="F17" r:id="rId79" xr:uid="{5D05AAA5-6C4E-4951-8A01-ED8966A74C6F}"/>
+    <hyperlink ref="H17" r:id="rId80" xr:uid="{F455D43D-0AE8-4F39-B8B8-A9E496C9515D}"/>
+    <hyperlink ref="F18" r:id="rId81" xr:uid="{5119747E-83D1-43AE-B78D-77BFA9310B65}"/>
+    <hyperlink ref="G18" r:id="rId82" xr:uid="{79EB751C-298E-437E-BEE6-FA6698B99FB9}"/>
+    <hyperlink ref="H18" r:id="rId83" xr:uid="{0509DA5B-CB9D-43F8-8168-2BABDCB86042}"/>
+    <hyperlink ref="I18" r:id="rId84" xr:uid="{ECC362EA-7284-4D5F-961E-DDABCD606149}"/>
+    <hyperlink ref="J18" r:id="rId85" xr:uid="{C4D0C97C-3218-467C-949C-4AE1EBBC383C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Arabic names added to the indoor plants sheet
</commit_message>
<xml_diff>
--- a/data/Locations.xlsx
+++ b/data/Locations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\landscapingUOB-api\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A98D4AEE-B9BD-48DF-9BC7-7CE0E90A0793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB9B7452-C7BB-4755-84F4-39E4B7FBFD27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="160">
   <si>
     <t>Location type</t>
   </si>
@@ -191,24 +191,9 @@
     <t>https://i.postimg.cc/bvBKCNZ0/S38-1.jpg</t>
   </si>
   <si>
-    <t>S39</t>
-  </si>
-  <si>
-    <t xml:space="preserve">College of Law </t>
-  </si>
-  <si>
     <t>https://i.postimg.cc/26jVwGBL/S39.jpg</t>
   </si>
   <si>
-    <t>S39A</t>
-  </si>
-  <si>
-    <t>Legal Clinic Office</t>
-  </si>
-  <si>
-    <t>https://i.postimg.cc/y8mhfRd7/S39A.jpg</t>
-  </si>
-  <si>
     <t>S4</t>
   </si>
   <si>
@@ -341,18 +326,6 @@
     <t>https://i.postimg.cc/wx1GwWdH/S54-2.jpg</t>
   </si>
   <si>
-    <t>S56</t>
-  </si>
-  <si>
-    <t>Trade Workshop</t>
-  </si>
-  <si>
-    <t>https://i.postimg.cc/mrYRjcZ6/S56-2.jpg</t>
-  </si>
-  <si>
-    <t>S57</t>
-  </si>
-  <si>
     <t>Business Incubator Center</t>
   </si>
   <si>
@@ -368,12 +341,6 @@
     <t>Infrastructure</t>
   </si>
   <si>
-    <t>S1</t>
-  </si>
-  <si>
-    <t>Boundary Wall</t>
-  </si>
-  <si>
     <t>Facilities</t>
   </si>
   <si>
@@ -522,6 +489,33 @@
   </si>
   <si>
     <t>https://i.postimg.cc/wxC15vc6/S39-3.jpg</t>
+  </si>
+  <si>
+    <t>S56, S57</t>
+  </si>
+  <si>
+    <t>S39, S39A</t>
+  </si>
+  <si>
+    <t>College of Law, Legal Clinic Office</t>
+  </si>
+  <si>
+    <t>Boundary Wall - Main Gate</t>
+  </si>
+  <si>
+    <t>Boundary Wall - Western Gate</t>
+  </si>
+  <si>
+    <t>Boundary Wall - Eastern Gate</t>
+  </si>
+  <si>
+    <t>Gate 1</t>
+  </si>
+  <si>
+    <t>Gate 2</t>
+  </si>
+  <si>
+    <t>Gate 3</t>
   </si>
 </sst>
 </file>
@@ -557,18 +551,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -578,13 +566,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFE163"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -620,19 +602,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -914,7 +898,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.90625" customWidth="1"/>
@@ -934,7 +918,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -943,22 +927,22 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -977,20 +961,20 @@
       <c r="E2">
         <v>699</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="H2" s="13" t="s">
-        <v>142</v>
-      </c>
-      <c r="I2" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="J2" s="13" t="s">
-        <v>144</v>
+      <c r="G2" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -1009,11 +993,11 @@
       <c r="E3">
         <v>600</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="13" t="s">
-        <v>145</v>
+      <c r="G3" s="8" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -1032,11 +1016,11 @@
       <c r="E4">
         <v>350</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="13" t="s">
-        <v>146</v>
+      <c r="G4" s="8" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -1055,11 +1039,11 @@
       <c r="E5">
         <v>186</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="13" t="s">
-        <v>147</v>
+      <c r="G5" s="8" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -1078,14 +1062,14 @@
       <c r="E6">
         <v>77</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="G6" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="H6" s="13" t="s">
-        <v>149</v>
+      <c r="G6" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -1104,7 +1088,7 @@
       <c r="E7">
         <v>330</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="8" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1124,7 +1108,7 @@
       <c r="E8">
         <v>280</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="8" t="s">
         <v>24</v>
       </c>
     </row>
@@ -1144,7 +1128,7 @@
       <c r="E9">
         <v>270</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="8" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1164,7 +1148,7 @@
       <c r="E10">
         <v>120</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="8" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1184,11 +1168,11 @@
       <c r="E11">
         <v>440</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="13" t="s">
-        <v>152</v>
+      <c r="G11" s="8" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -1207,7 +1191,7 @@
       <c r="E12">
         <v>105</v>
       </c>
-      <c r="F12" s="13" t="s">
+      <c r="F12" s="8" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1227,7 +1211,7 @@
       <c r="E13">
         <v>1050</v>
       </c>
-      <c r="F13" s="13" t="s">
+      <c r="F13" s="8" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1247,7 +1231,7 @@
       <c r="E14">
         <v>80</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="F14" s="8" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1267,7 +1251,7 @@
       <c r="E15">
         <v>145</v>
       </c>
-      <c r="F15" s="13" t="s">
+      <c r="F15" s="8" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1282,19 +1266,19 @@
         <v>47</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="E16">
         <v>1350</v>
       </c>
-      <c r="F16" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="G16" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="H16" s="13" t="s">
-        <v>155</v>
+      <c r="F16" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -1313,14 +1297,14 @@
       <c r="E17">
         <v>175</v>
       </c>
-      <c r="F17" s="13" t="s">
+      <c r="F17" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="G17" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="H17" s="13" t="s">
-        <v>157</v>
+      <c r="G17" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -1328,48 +1312,48 @@
         <v>3</v>
       </c>
       <c r="B18" t="s">
+        <v>152</v>
+      </c>
+      <c r="C18" t="s">
+        <v>153</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="C18" t="s">
-        <v>52</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>53</v>
       </c>
       <c r="E18">
         <v>1000</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="F18" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" t="s">
         <v>53</v>
       </c>
-      <c r="G18" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="H18" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="I18" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="J18" s="13" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B19" s="7" t="s">
+      <c r="D19" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="E19" s="7">
-        <v>1000</v>
+      <c r="E19">
+        <v>350</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
@@ -1377,16 +1361,16 @@
         <v>3</v>
       </c>
       <c r="B20" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C20" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>59</v>
-      </c>
       <c r="E20">
-        <v>350</v>
+        <v>464</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
@@ -1394,16 +1378,16 @@
         <v>3</v>
       </c>
       <c r="B21" t="s">
+        <v>58</v>
+      </c>
+      <c r="C21" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C21" t="s">
-        <v>61</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>62</v>
-      </c>
       <c r="E21">
-        <v>464</v>
+        <v>310</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
@@ -1411,16 +1395,16 @@
         <v>3</v>
       </c>
       <c r="B22" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" t="s">
+        <v>62</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C22" t="s">
-        <v>64</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>65</v>
-      </c>
       <c r="E22">
-        <v>310</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
@@ -1428,16 +1412,16 @@
         <v>3</v>
       </c>
       <c r="B23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C23" t="s">
-        <v>67</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>68</v>
-      </c>
       <c r="E23">
-        <v>195</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
@@ -1445,16 +1429,16 @@
         <v>3</v>
       </c>
       <c r="B24" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24" t="s">
+        <v>68</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C24" t="s">
-        <v>70</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>71</v>
-      </c>
       <c r="E24">
-        <v>45</v>
+        <v>180</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
@@ -1462,73 +1446,73 @@
         <v>3</v>
       </c>
       <c r="B25" t="s">
+        <v>70</v>
+      </c>
+      <c r="C25" t="s">
+        <v>71</v>
+      </c>
+      <c r="D25" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C25" t="s">
+      <c r="E25">
+        <v>90</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="H25" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>3</v>
+      </c>
+      <c r="B26" t="s">
         <v>73</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="C26" t="s">
         <v>74</v>
       </c>
-      <c r="E25">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>3</v>
-      </c>
-      <c r="B26" t="s">
+      <c r="D26" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C26" t="s">
+      <c r="E26">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" s="6" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="C27" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="E26">
-        <v>90</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="G26" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="H26" s="13" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>3</v>
-      </c>
-      <c r="B27" t="s">
+      <c r="D27" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C27" t="s">
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" t="s">
         <v>79</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="C28" t="s">
         <v>80</v>
       </c>
-      <c r="E27">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B28" s="7" t="s">
+      <c r="D28" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C28" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>83</v>
+      <c r="E28">
+        <v>399</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
@@ -1536,16 +1520,16 @@
         <v>3</v>
       </c>
       <c r="B29" t="s">
+        <v>82</v>
+      </c>
+      <c r="C29" t="s">
+        <v>83</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="C29" t="s">
-        <v>85</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>86</v>
-      </c>
       <c r="E29">
-        <v>399</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
@@ -1553,16 +1537,16 @@
         <v>3</v>
       </c>
       <c r="B30" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" t="s">
+        <v>86</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="C30" t="s">
-        <v>88</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>89</v>
-      </c>
       <c r="E30">
-        <v>163</v>
+        <v>194</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.35">
@@ -1570,16 +1554,16 @@
         <v>3</v>
       </c>
       <c r="B31" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C31" t="s">
-        <v>91</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="E31">
-        <v>194</v>
+        <v>373</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
@@ -1587,164 +1571,154 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
+        <v>91</v>
+      </c>
+      <c r="C32" t="s">
+        <v>83</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E32">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B33" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C33" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D33" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="E32">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>3</v>
-      </c>
-      <c r="B33" t="s">
+      <c r="E33" s="6">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="C34" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="C33" t="s">
-        <v>88</v>
-      </c>
-      <c r="D33" s="5" t="s">
+      <c r="D34" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="E33">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B34" s="7" t="s">
+      <c r="E34" s="9">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>3</v>
+      </c>
+      <c r="B35" t="s">
         <v>98</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C35" t="s">
         <v>99</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="D35" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="E35">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A36" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E34" s="7">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="E35" s="7">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="E36" s="7">
-        <v>205</v>
+      <c r="B36" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="C36" t="s">
+        <v>154</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="E36">
+        <v>142</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>3</v>
+      <c r="A37" s="3" t="s">
+        <v>100</v>
       </c>
       <c r="B37" t="s">
-        <v>107</v>
+        <v>158</v>
       </c>
       <c r="C37" t="s">
-        <v>108</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="E37">
-        <v>350</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="D37" s="12"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>110</v>
+        <v>100</v>
+      </c>
+      <c r="B38" t="s">
+        <v>159</v>
       </c>
       <c r="C38" t="s">
-        <v>111</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="E38">
-        <v>142</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="D38" s="12"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="B39" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C39" t="s">
-        <v>128</v>
-      </c>
-      <c r="D39" s="9"/>
+        <v>117</v>
+      </c>
+      <c r="D39" s="12"/>
       <c r="E39">
         <v>1300</v>
       </c>
     </row>
-    <row r="40" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="E40" s="7">
+    <row r="40" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E40" s="6">
         <v>600</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="B41" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="E41">
         <v>5300</v>
@@ -1752,16 +1726,16 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="B42" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="C42" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="E42">
         <v>16500</v>
@@ -1769,16 +1743,16 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="B43" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="C43" t="s">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="E43">
         <v>16500</v>
@@ -1786,7 +1760,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="B44" t="s">
         <v>25</v>
@@ -1803,131 +1777,114 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="B45" t="s">
+        <v>152</v>
+      </c>
+      <c r="C45" t="s">
+        <v>153</v>
+      </c>
+      <c r="D45" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="C45" t="s">
-        <v>52</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>53</v>
       </c>
       <c r="E45">
         <v>400</v>
       </c>
     </row>
-    <row r="46" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="B46" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C46" s="7" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>116</v>
+      </c>
+      <c r="B46" t="s">
         <v>55</v>
       </c>
-      <c r="D46" s="8" t="s">
+      <c r="C46" t="s">
         <v>56</v>
       </c>
-      <c r="E46" s="7">
-        <v>400</v>
+      <c r="D46" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E46">
+        <v>704</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="B47" t="s">
+        <v>58</v>
+      </c>
+      <c r="C47" t="s">
+        <v>59</v>
+      </c>
+      <c r="D47" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C47" t="s">
-        <v>61</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>62</v>
-      </c>
       <c r="E47">
-        <v>704</v>
+        <v>602</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="B48" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="C48" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="E48">
-        <v>602</v>
+        <v>128</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="B49" t="s">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="C49" t="s">
-        <v>82</v>
+        <v>113</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="E49">
-        <v>128</v>
+        <v>825</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>127</v>
-      </c>
-      <c r="B50" t="s">
-        <v>123</v>
+        <v>3</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>10</v>
       </c>
       <c r="C50" t="s">
-        <v>124</v>
-      </c>
-      <c r="D50" s="5" t="s">
-        <v>125</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="D50" s="10"/>
       <c r="E50">
-        <v>825</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>3</v>
-      </c>
-      <c r="B51" s="12" t="s">
-        <v>10</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="B51" s="11"/>
       <c r="C51" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="D51" s="10"/>
       <c r="E51">
-        <v>2550</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>130</v>
-      </c>
-      <c r="B52" s="11"/>
-      <c r="C52" t="s">
-        <v>131</v>
-      </c>
-      <c r="D52" s="10"/>
-      <c r="E52">
         <v>13500</v>
       </c>
     </row>
@@ -1963,71 +1920,68 @@
     <hyperlink ref="D6" r:id="rId18" xr:uid="{705A06BF-AD9E-4AEF-8BEC-6580A15197D6}"/>
     <hyperlink ref="D44" r:id="rId19" xr:uid="{F581F61C-236D-49A3-AE06-C2A7FF968C89}"/>
     <hyperlink ref="D45" r:id="rId20" xr:uid="{BB91F514-736D-4FC9-A32E-788A20E577B9}"/>
-    <hyperlink ref="D46" r:id="rId21" xr:uid="{7EBDAD46-1A5B-4B2C-AF3D-61F18C3E275F}"/>
-    <hyperlink ref="D47" r:id="rId22" xr:uid="{A36D56AA-7C90-4154-A870-DA9409189D1F}"/>
-    <hyperlink ref="D48" r:id="rId23" xr:uid="{00DDF648-5623-4E1D-8FC4-42D38FAEE4CA}"/>
-    <hyperlink ref="D49" r:id="rId24" xr:uid="{77EAAAD6-086C-4DCF-9B24-E59430A2E2FB}"/>
-    <hyperlink ref="D50" r:id="rId25" xr:uid="{CE8A3876-BF7A-4C23-95FB-161481F8F980}"/>
-    <hyperlink ref="F26" r:id="rId26" xr:uid="{E4CD215B-218A-44EC-9945-5F6AD197B3B2}"/>
-    <hyperlink ref="G26" r:id="rId27" xr:uid="{522CE0D5-7681-455E-9A32-6774CD570260}"/>
-    <hyperlink ref="H26" r:id="rId28" xr:uid="{A440C7F8-BC12-4ED8-80D1-5687F587FDDF}"/>
-    <hyperlink ref="G2" r:id="rId29" xr:uid="{E92EE150-871A-439E-974B-FA2049C8CA38}"/>
-    <hyperlink ref="H2" r:id="rId30" xr:uid="{03D46786-9004-478B-A395-4AA7EF082A56}"/>
-    <hyperlink ref="I2" r:id="rId31" xr:uid="{57A7AAAC-E898-44F4-A3B0-AF97E1EBFE69}"/>
-    <hyperlink ref="J2" r:id="rId32" xr:uid="{ACBBE8A2-CC26-4054-A6DA-6E5C07960AD1}"/>
-    <hyperlink ref="F3" r:id="rId33" xr:uid="{29114336-215A-43FA-8297-CDDD761C1501}"/>
-    <hyperlink ref="G3" r:id="rId34" xr:uid="{0AE835A0-8DDB-4A91-8176-2AFF9C2AEA07}"/>
-    <hyperlink ref="F4" r:id="rId35" xr:uid="{9F1D3B58-9986-4688-ABF5-8FF2375FBF82}"/>
-    <hyperlink ref="G4" r:id="rId36" xr:uid="{6CB43155-6638-4798-B491-DB6FA525EB50}"/>
-    <hyperlink ref="F5" r:id="rId37" xr:uid="{7DCFF457-0664-4586-B064-437E516400A0}"/>
-    <hyperlink ref="G5" r:id="rId38" xr:uid="{343CFCD0-DE46-476D-8E81-253A8E3B316C}"/>
-    <hyperlink ref="F6" r:id="rId39" xr:uid="{3EC21E9D-842C-4CB8-B811-D23F2C778BF7}"/>
-    <hyperlink ref="G6" r:id="rId40" xr:uid="{33FCB128-9197-43CE-8CB7-FE8F3059BE4F}"/>
-    <hyperlink ref="H6" r:id="rId41" xr:uid="{1F8966A1-2290-4CEF-BB02-FC990CD8D791}"/>
-    <hyperlink ref="F7" r:id="rId42" xr:uid="{423CFF82-45DF-4D68-BB50-979F20779C0F}"/>
-    <hyperlink ref="F8" r:id="rId43" xr:uid="{E5CBA92A-AB4F-478A-9CFE-9419577F0ED5}"/>
-    <hyperlink ref="F10" r:id="rId44" xr:uid="{EB116F53-35BE-4168-A3B3-A6B7F3013480}"/>
-    <hyperlink ref="F9" r:id="rId45" xr:uid="{AAFC07D3-B9CC-483D-8F88-4D08FD7ED6B1}"/>
-    <hyperlink ref="F11" r:id="rId46" xr:uid="{E9FA1CD4-77B0-4337-B7D9-41FF5FAF8D5C}"/>
-    <hyperlink ref="G11" r:id="rId47" xr:uid="{44406BDF-4864-4DEE-8D3F-960771AC5EEA}"/>
-    <hyperlink ref="F12" r:id="rId48" xr:uid="{A2470070-51EF-4670-833B-8D482C601671}"/>
-    <hyperlink ref="F13" r:id="rId49" xr:uid="{4D4972B4-0A24-4319-992B-3F7B5C4CCDCE}"/>
-    <hyperlink ref="F14" r:id="rId50" xr:uid="{AE1ACB1F-F85D-4CF3-AC72-FD2F25C8E4B2}"/>
-    <hyperlink ref="D22" r:id="rId51" xr:uid="{6E85802D-CC4C-4BD4-83ED-55100DE115BA}"/>
-    <hyperlink ref="D37" r:id="rId52" xr:uid="{6683E2F8-FB9A-4014-9996-7FEAAC683B93}"/>
-    <hyperlink ref="D35" r:id="rId53" xr:uid="{368C86F0-6C72-4FCF-9F6B-86FBA36B83AF}"/>
-    <hyperlink ref="D38" r:id="rId54" xr:uid="{6AF44C4C-D5AE-4BD7-8C44-C3D0460467C0}"/>
-    <hyperlink ref="D20" r:id="rId55" xr:uid="{80ECF8CD-7A79-402A-B5EC-F9BA63C3B50A}"/>
-    <hyperlink ref="D34" r:id="rId56" xr:uid="{E93DF50E-6385-47B4-B2C7-B9246E51EFC3}"/>
-    <hyperlink ref="D23" r:id="rId57" xr:uid="{13D49606-5D63-4601-9617-2606341647E2}"/>
-    <hyperlink ref="D24" r:id="rId58" xr:uid="{D83D9F73-94C9-4362-9F33-9764794F83C7}"/>
-    <hyperlink ref="D30" r:id="rId59" xr:uid="{7CB307A7-AD29-447B-B87B-FDF01946BA4A}"/>
-    <hyperlink ref="D29" r:id="rId60" xr:uid="{45AB639A-6A68-47E6-820F-5AE96EF37CCE}"/>
-    <hyperlink ref="D28" r:id="rId61" xr:uid="{A6B3F117-56EC-4411-89C5-2B81B32C6D2F}"/>
-    <hyperlink ref="D32" r:id="rId62" xr:uid="{0BEBBA09-865C-426C-A4B4-4F2481A2A4E8}"/>
-    <hyperlink ref="D26" r:id="rId63" xr:uid="{EFEDD41E-1E02-461C-9393-AD2ACCBC2A60}"/>
-    <hyperlink ref="D27" r:id="rId64" xr:uid="{40D3F8D6-8B9A-4507-8102-4BFB0D9B2580}"/>
-    <hyperlink ref="D21" r:id="rId65" xr:uid="{5BA1C18C-D565-4734-9906-9C0A7DC7BFEA}"/>
-    <hyperlink ref="D36" r:id="rId66" xr:uid="{E63D41F9-5B08-43E0-8053-0724E6D37B6B}"/>
-    <hyperlink ref="D18" r:id="rId67" xr:uid="{2D6E9249-18AB-4397-B0F5-437EFBC6F332}"/>
-    <hyperlink ref="D17" r:id="rId68" xr:uid="{6EEDF604-934E-4BBF-844F-1CBB5949AF7F}"/>
-    <hyperlink ref="D16" r:id="rId69" xr:uid="{B21EE433-AA31-44F8-A2B5-B896D27134D4}"/>
-    <hyperlink ref="D33" r:id="rId70" xr:uid="{8D11C5C3-9012-49EE-A7E5-072DFCD7E4CB}"/>
-    <hyperlink ref="D31" r:id="rId71" xr:uid="{99947C2E-DEFB-4F3D-B10B-4C51E1A36A2A}"/>
-    <hyperlink ref="D19" r:id="rId72" xr:uid="{7BE3DA68-E823-4B16-885B-945823145A4E}"/>
-    <hyperlink ref="D25" r:id="rId73" xr:uid="{CA6F2ACE-9B39-4D45-9C20-19A5DB6D12CA}"/>
-    <hyperlink ref="F15" r:id="rId74" xr:uid="{C35D8A0A-F10A-40F3-A7C3-C5AA6BBB28B5}"/>
-    <hyperlink ref="F16" r:id="rId75" xr:uid="{AEA8472C-440C-4C92-8A77-FEF9C839BF0D}"/>
-    <hyperlink ref="G16" r:id="rId76" xr:uid="{D288EC2B-5C10-4124-87EF-58A40C745452}"/>
-    <hyperlink ref="H16" r:id="rId77" xr:uid="{AB6F38F4-9CD4-49B8-9315-6A116F3871B3}"/>
-    <hyperlink ref="G17" r:id="rId78" xr:uid="{A5B70704-22DA-478D-9DD9-DCC7AA836C2E}"/>
-    <hyperlink ref="F17" r:id="rId79" xr:uid="{5D05AAA5-6C4E-4951-8A01-ED8966A74C6F}"/>
-    <hyperlink ref="H17" r:id="rId80" xr:uid="{F455D43D-0AE8-4F39-B8B8-A9E496C9515D}"/>
-    <hyperlink ref="F18" r:id="rId81" xr:uid="{5119747E-83D1-43AE-B78D-77BFA9310B65}"/>
-    <hyperlink ref="G18" r:id="rId82" xr:uid="{79EB751C-298E-437E-BEE6-FA6698B99FB9}"/>
-    <hyperlink ref="H18" r:id="rId83" xr:uid="{0509DA5B-CB9D-43F8-8168-2BABDCB86042}"/>
-    <hyperlink ref="I18" r:id="rId84" xr:uid="{ECC362EA-7284-4D5F-961E-DDABCD606149}"/>
-    <hyperlink ref="J18" r:id="rId85" xr:uid="{C4D0C97C-3218-467C-949C-4AE1EBBC383C}"/>
+    <hyperlink ref="D46" r:id="rId21" xr:uid="{A36D56AA-7C90-4154-A870-DA9409189D1F}"/>
+    <hyperlink ref="D47" r:id="rId22" xr:uid="{00DDF648-5623-4E1D-8FC4-42D38FAEE4CA}"/>
+    <hyperlink ref="D48" r:id="rId23" xr:uid="{77EAAAD6-086C-4DCF-9B24-E59430A2E2FB}"/>
+    <hyperlink ref="D49" r:id="rId24" xr:uid="{CE8A3876-BF7A-4C23-95FB-161481F8F980}"/>
+    <hyperlink ref="F25" r:id="rId25" xr:uid="{E4CD215B-218A-44EC-9945-5F6AD197B3B2}"/>
+    <hyperlink ref="G25" r:id="rId26" xr:uid="{522CE0D5-7681-455E-9A32-6774CD570260}"/>
+    <hyperlink ref="H25" r:id="rId27" xr:uid="{A440C7F8-BC12-4ED8-80D1-5687F587FDDF}"/>
+    <hyperlink ref="G2" r:id="rId28" xr:uid="{E92EE150-871A-439E-974B-FA2049C8CA38}"/>
+    <hyperlink ref="H2" r:id="rId29" xr:uid="{03D46786-9004-478B-A395-4AA7EF082A56}"/>
+    <hyperlink ref="I2" r:id="rId30" xr:uid="{57A7AAAC-E898-44F4-A3B0-AF97E1EBFE69}"/>
+    <hyperlink ref="J2" r:id="rId31" xr:uid="{ACBBE8A2-CC26-4054-A6DA-6E5C07960AD1}"/>
+    <hyperlink ref="F3" r:id="rId32" xr:uid="{29114336-215A-43FA-8297-CDDD761C1501}"/>
+    <hyperlink ref="G3" r:id="rId33" xr:uid="{0AE835A0-8DDB-4A91-8176-2AFF9C2AEA07}"/>
+    <hyperlink ref="F4" r:id="rId34" xr:uid="{9F1D3B58-9986-4688-ABF5-8FF2375FBF82}"/>
+    <hyperlink ref="G4" r:id="rId35" xr:uid="{6CB43155-6638-4798-B491-DB6FA525EB50}"/>
+    <hyperlink ref="F5" r:id="rId36" xr:uid="{7DCFF457-0664-4586-B064-437E516400A0}"/>
+    <hyperlink ref="G5" r:id="rId37" xr:uid="{343CFCD0-DE46-476D-8E81-253A8E3B316C}"/>
+    <hyperlink ref="F6" r:id="rId38" xr:uid="{3EC21E9D-842C-4CB8-B811-D23F2C778BF7}"/>
+    <hyperlink ref="G6" r:id="rId39" xr:uid="{33FCB128-9197-43CE-8CB7-FE8F3059BE4F}"/>
+    <hyperlink ref="H6" r:id="rId40" xr:uid="{1F8966A1-2290-4CEF-BB02-FC990CD8D791}"/>
+    <hyperlink ref="F7" r:id="rId41" xr:uid="{423CFF82-45DF-4D68-BB50-979F20779C0F}"/>
+    <hyperlink ref="F8" r:id="rId42" xr:uid="{E5CBA92A-AB4F-478A-9CFE-9419577F0ED5}"/>
+    <hyperlink ref="F10" r:id="rId43" xr:uid="{EB116F53-35BE-4168-A3B3-A6B7F3013480}"/>
+    <hyperlink ref="F9" r:id="rId44" xr:uid="{AAFC07D3-B9CC-483D-8F88-4D08FD7ED6B1}"/>
+    <hyperlink ref="F11" r:id="rId45" xr:uid="{E9FA1CD4-77B0-4337-B7D9-41FF5FAF8D5C}"/>
+    <hyperlink ref="G11" r:id="rId46" xr:uid="{44406BDF-4864-4DEE-8D3F-960771AC5EEA}"/>
+    <hyperlink ref="F12" r:id="rId47" xr:uid="{A2470070-51EF-4670-833B-8D482C601671}"/>
+    <hyperlink ref="F13" r:id="rId48" xr:uid="{4D4972B4-0A24-4319-992B-3F7B5C4CCDCE}"/>
+    <hyperlink ref="F14" r:id="rId49" xr:uid="{AE1ACB1F-F85D-4CF3-AC72-FD2F25C8E4B2}"/>
+    <hyperlink ref="D21" r:id="rId50" xr:uid="{6E85802D-CC4C-4BD4-83ED-55100DE115BA}"/>
+    <hyperlink ref="D35" r:id="rId51" xr:uid="{6683E2F8-FB9A-4014-9996-7FEAAC683B93}"/>
+    <hyperlink ref="D36" r:id="rId52" xr:uid="{6AF44C4C-D5AE-4BD7-8C44-C3D0460467C0}"/>
+    <hyperlink ref="D19" r:id="rId53" xr:uid="{80ECF8CD-7A79-402A-B5EC-F9BA63C3B50A}"/>
+    <hyperlink ref="D33" r:id="rId54" xr:uid="{E93DF50E-6385-47B4-B2C7-B9246E51EFC3}"/>
+    <hyperlink ref="D22" r:id="rId55" xr:uid="{13D49606-5D63-4601-9617-2606341647E2}"/>
+    <hyperlink ref="D23" r:id="rId56" xr:uid="{D83D9F73-94C9-4362-9F33-9764794F83C7}"/>
+    <hyperlink ref="D29" r:id="rId57" xr:uid="{7CB307A7-AD29-447B-B87B-FDF01946BA4A}"/>
+    <hyperlink ref="D28" r:id="rId58" xr:uid="{45AB639A-6A68-47E6-820F-5AE96EF37CCE}"/>
+    <hyperlink ref="D27" r:id="rId59" xr:uid="{A6B3F117-56EC-4411-89C5-2B81B32C6D2F}"/>
+    <hyperlink ref="D31" r:id="rId60" xr:uid="{0BEBBA09-865C-426C-A4B4-4F2481A2A4E8}"/>
+    <hyperlink ref="D25" r:id="rId61" xr:uid="{EFEDD41E-1E02-461C-9393-AD2ACCBC2A60}"/>
+    <hyperlink ref="D26" r:id="rId62" xr:uid="{40D3F8D6-8B9A-4507-8102-4BFB0D9B2580}"/>
+    <hyperlink ref="D20" r:id="rId63" xr:uid="{5BA1C18C-D565-4734-9906-9C0A7DC7BFEA}"/>
+    <hyperlink ref="D34" r:id="rId64" xr:uid="{E63D41F9-5B08-43E0-8053-0724E6D37B6B}"/>
+    <hyperlink ref="D18" r:id="rId65" xr:uid="{2D6E9249-18AB-4397-B0F5-437EFBC6F332}"/>
+    <hyperlink ref="D17" r:id="rId66" xr:uid="{6EEDF604-934E-4BBF-844F-1CBB5949AF7F}"/>
+    <hyperlink ref="D16" r:id="rId67" xr:uid="{B21EE433-AA31-44F8-A2B5-B896D27134D4}"/>
+    <hyperlink ref="D32" r:id="rId68" xr:uid="{8D11C5C3-9012-49EE-A7E5-072DFCD7E4CB}"/>
+    <hyperlink ref="D30" r:id="rId69" xr:uid="{99947C2E-DEFB-4F3D-B10B-4C51E1A36A2A}"/>
+    <hyperlink ref="D24" r:id="rId70" xr:uid="{CA6F2ACE-9B39-4D45-9C20-19A5DB6D12CA}"/>
+    <hyperlink ref="F15" r:id="rId71" xr:uid="{C35D8A0A-F10A-40F3-A7C3-C5AA6BBB28B5}"/>
+    <hyperlink ref="F16" r:id="rId72" xr:uid="{AEA8472C-440C-4C92-8A77-FEF9C839BF0D}"/>
+    <hyperlink ref="G16" r:id="rId73" xr:uid="{D288EC2B-5C10-4124-87EF-58A40C745452}"/>
+    <hyperlink ref="H16" r:id="rId74" xr:uid="{AB6F38F4-9CD4-49B8-9315-6A116F3871B3}"/>
+    <hyperlink ref="G17" r:id="rId75" xr:uid="{A5B70704-22DA-478D-9DD9-DCC7AA836C2E}"/>
+    <hyperlink ref="F17" r:id="rId76" xr:uid="{5D05AAA5-6C4E-4951-8A01-ED8966A74C6F}"/>
+    <hyperlink ref="H17" r:id="rId77" xr:uid="{F455D43D-0AE8-4F39-B8B8-A9E496C9515D}"/>
+    <hyperlink ref="F18" r:id="rId78" xr:uid="{5119747E-83D1-43AE-B78D-77BFA9310B65}"/>
+    <hyperlink ref="G18" r:id="rId79" xr:uid="{79EB751C-298E-437E-BEE6-FA6698B99FB9}"/>
+    <hyperlink ref="H18" r:id="rId80" xr:uid="{0509DA5B-CB9D-43F8-8168-2BABDCB86042}"/>
+    <hyperlink ref="I18" r:id="rId81" xr:uid="{ECC362EA-7284-4D5F-961E-DDABCD606149}"/>
+    <hyperlink ref="J18" r:id="rId82" xr:uid="{C4D0C97C-3218-467C-949C-4AE1EBBC383C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>